<commit_message>
Radar: datos del 2026-08-31
</commit_message>
<xml_diff>
--- a/web/descargas/licitaciones.xlsx
+++ b/web/descargas/licitaciones.xlsx
@@ -412,7 +412,7 @@
         <v>46265.625</v>
       </c>
       <c r="J2" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" s="3">
         <v>4000000.0</v>
@@ -501,7 +501,7 @@
         <v>46265.625</v>
       </c>
       <c r="J3" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" s="3">
         <v>6000000.0</v>
@@ -589,7 +589,7 @@
         <v>46265.625</v>
       </c>
       <c r="J4" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" s="3"/>
       <c r="L4" s="0" t="inlineStr">
@@ -682,7 +682,7 @@
         <v>46265.625</v>
       </c>
       <c r="J5" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" s="3"/>
       <c r="L5" s="0" t="inlineStr">
@@ -775,7 +775,7 @@
         <v>46265.625</v>
       </c>
       <c r="J6" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" s="3"/>
       <c r="L6" s="0" t="inlineStr">
@@ -875,7 +875,7 @@
         <v>46265.625</v>
       </c>
       <c r="J7" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" s="3">
         <v>15000000.0</v>
@@ -970,7 +970,7 @@
         <v>46265.625</v>
       </c>
       <c r="J8" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" s="3">
         <v>14000000.0</v>
@@ -1065,7 +1065,7 @@
         <v>46265.625694</v>
       </c>
       <c r="J9" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" s="3"/>
       <c r="L9" s="0" t="inlineStr">
@@ -1159,7 +1159,7 @@
         <v>46265.625694</v>
       </c>
       <c r="J10" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" s="3">
         <v>4500000.0</v>
@@ -1242,7 +1242,7 @@
         <v>46265.625694</v>
       </c>
       <c r="J11" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" s="3">
         <v>42000000.0</v>
@@ -1337,7 +1337,7 @@
         <v>46265.631944</v>
       </c>
       <c r="J12" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" s="3">
         <v>12000.0</v>
@@ -1436,7 +1436,7 @@
         <v>46265.645833</v>
       </c>
       <c r="J13" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13" s="3">
         <v>49800000.0</v>
@@ -1531,7 +1531,7 @@
         <v>46265.645833</v>
       </c>
       <c r="J14" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14" s="3"/>
       <c r="L14" s="0" t="inlineStr">
@@ -1624,7 +1624,7 @@
         <v>46265.646528</v>
       </c>
       <c r="J15" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" s="3">
         <v>3000000.0</v>
@@ -1719,7 +1719,7 @@
         <v>46265.666667</v>
       </c>
       <c r="J16" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K16" s="3">
         <v>175000000.0</v>
@@ -1814,7 +1814,7 @@
         <v>46265.666667</v>
       </c>
       <c r="J17" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K17" s="3">
         <v>4522419.0</v>
@@ -1901,7 +1901,7 @@
         <v>46265.708333</v>
       </c>
       <c r="J18" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" s="3">
         <v>434042600.0</v>
@@ -1998,7 +1998,7 @@
         <v>46265.854167</v>
       </c>
       <c r="J19" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K19" s="3">
         <v>4526046.0</v>
@@ -2085,7 +2085,7 @@
         <v>46266.604167</v>
       </c>
       <c r="J20" s="0">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K20" s="3"/>
       <c r="L20" s="0" t="inlineStr">
@@ -2178,7 +2178,7 @@
         <v>46266.625</v>
       </c>
       <c r="J21" s="0">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K21" s="3"/>
       <c r="L21" s="0" t="inlineStr">
@@ -2271,7 +2271,7 @@
         <v>46266.631944</v>
       </c>
       <c r="J22" s="0">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K22" s="3">
         <v>33150.0</v>
@@ -2366,7 +2366,7 @@
         <v>46266.666667</v>
       </c>
       <c r="J23" s="0">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K23" s="3">
         <v>12154650.0</v>
@@ -2460,7 +2460,7 @@
         <v>46266.666667</v>
       </c>
       <c r="J24" s="0">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K24" s="3">
         <v>190000000.0</v>
@@ -2555,7 +2555,7 @@
         <v>46266.692361</v>
       </c>
       <c r="J25" s="0">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K25" s="3"/>
       <c r="L25" s="0" t="inlineStr">
@@ -2648,7 +2648,7 @@
         <v>46267.625</v>
       </c>
       <c r="J26" s="0">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K26" s="3">
         <v>19800000.0</v>
@@ -2739,7 +2739,7 @@
         <v>46267.625</v>
       </c>
       <c r="J27" s="0">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K27" s="3"/>
       <c r="L27" s="0" t="inlineStr">
@@ -2832,7 +2832,7 @@
         <v>46267.645833</v>
       </c>
       <c r="J28" s="0">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K28" s="3">
         <v>22000000.0</v>
@@ -2927,7 +2927,7 @@
         <v>46267.708333</v>
       </c>
       <c r="J29" s="0">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K29" s="3">
         <v>15000000.0</v>
@@ -3018,7 +3018,7 @@
         <v>46267.709028</v>
       </c>
       <c r="J30" s="0">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K30" s="3"/>
       <c r="L30" s="0" t="inlineStr">
@@ -3116,7 +3116,7 @@
         <v>46267.749306</v>
       </c>
       <c r="J31" s="0">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K31" s="3">
         <v>250000000.0</v>
@@ -3211,7 +3211,7 @@
         <v>46268.500694</v>
       </c>
       <c r="J32" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K32" s="3">
         <v>70000000.0</v>
@@ -3307,7 +3307,7 @@
         <v>46268.600694</v>
       </c>
       <c r="J33" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K33" s="3">
         <v>10000000.0</v>
@@ -3406,7 +3406,7 @@
         <v>46268.600694</v>
       </c>
       <c r="J34" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K34" s="3">
         <v>32500000.0</v>
@@ -3505,7 +3505,7 @@
         <v>46268.625</v>
       </c>
       <c r="J35" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K35" s="3">
         <v>15000000.0</v>
@@ -3600,7 +3600,7 @@
         <v>46268.625</v>
       </c>
       <c r="J36" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K36" s="3">
         <v>269000000.0</v>
@@ -3702,7 +3702,7 @@
         <v>46268.625</v>
       </c>
       <c r="J37" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K37" s="3">
         <v>1989000.0</v>
@@ -3791,7 +3791,7 @@
         <v>46268.645833</v>
       </c>
       <c r="J38" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K38" s="3">
         <v>8000000.0</v>
@@ -3883,7 +3883,7 @@
         <v>46268.645833</v>
       </c>
       <c r="J39" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K39" s="3"/>
       <c r="L39" s="0" t="inlineStr">
@@ -3976,7 +3976,7 @@
         <v>46268.666667</v>
       </c>
       <c r="J40" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K40" s="3">
         <v>14000000.0</v>
@@ -4067,7 +4067,7 @@
         <v>46268.675</v>
       </c>
       <c r="J41" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K41" s="3"/>
       <c r="L41" s="0" t="inlineStr">
@@ -4156,7 +4156,7 @@
         <v>46268.708333</v>
       </c>
       <c r="J42" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K42" s="3">
         <v>202000000.0</v>
@@ -4247,7 +4247,7 @@
         <v>46268.75</v>
       </c>
       <c r="J43" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K43" s="3">
         <v>32000000.0</v>
@@ -4342,7 +4342,7 @@
         <v>46269.375</v>
       </c>
       <c r="J44" s="0">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K44" s="3">
         <v>13000000.0</v>
@@ -4437,7 +4437,7 @@
         <v>46269.5</v>
       </c>
       <c r="J45" s="0">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K45" s="3">
         <v>40856640.0</v>
@@ -4532,7 +4532,7 @@
         <v>46269.625</v>
       </c>
       <c r="J46" s="0">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K46" s="3">
         <v>2500000.0</v>
@@ -4619,7 +4619,7 @@
         <v>46269.625</v>
       </c>
       <c r="J47" s="0">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K47" s="3"/>
       <c r="L47" s="0" t="inlineStr">
@@ -4712,7 +4712,7 @@
         <v>46269.666667</v>
       </c>
       <c r="J48" s="0">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K48" s="3"/>
       <c r="L48" s="0" t="inlineStr">
@@ -4809,7 +4809,7 @@
         <v>46269.708333</v>
       </c>
       <c r="J49" s="0">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K49" s="3">
         <v>4000000.0</v>
@@ -4898,7 +4898,7 @@
         <v>46269.833333</v>
       </c>
       <c r="J50" s="0">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K50" s="3">
         <v>27000000.0</v>
@@ -4993,7 +4993,7 @@
         <v>46272.625</v>
       </c>
       <c r="J51" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K51" s="3">
         <v>60000000.0</v>
@@ -5088,7 +5088,7 @@
         <v>46272.625</v>
       </c>
       <c r="J52" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K52" s="3">
         <v>16000000.0</v>
@@ -5179,7 +5179,7 @@
         <v>46272.625</v>
       </c>
       <c r="J53" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K53" s="3"/>
       <c r="L53" s="0" t="inlineStr">
@@ -5272,7 +5272,7 @@
         <v>46272.625</v>
       </c>
       <c r="J54" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K54" s="3">
         <v>4728.0</v>
@@ -5367,7 +5367,7 @@
         <v>46272.625694</v>
       </c>
       <c r="J55" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K55" s="3"/>
       <c r="L55" s="0" t="inlineStr">
@@ -5464,7 +5464,7 @@
         <v>46272.625694</v>
       </c>
       <c r="J56" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K56" s="3"/>
       <c r="L56" s="0" t="inlineStr">
@@ -5553,7 +5553,7 @@
         <v>46272.63125</v>
       </c>
       <c r="J57" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K57" s="3">
         <v>14000000.0</v>
@@ -5649,7 +5649,7 @@
         <v>46272.631944</v>
       </c>
       <c r="J58" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K58" s="3"/>
       <c r="L58" s="0" t="inlineStr">
@@ -5742,7 +5742,7 @@
         <v>46272.645833</v>
       </c>
       <c r="J59" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K59" s="3">
         <v>11300000.0</v>
@@ -5841,7 +5841,7 @@
         <v>46272.645833</v>
       </c>
       <c r="J60" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K60" s="3">
         <v>21500000.0</v>
@@ -5940,7 +5940,7 @@
         <v>46272.666667</v>
       </c>
       <c r="J61" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K61" s="3">
         <v>29790000.0</v>
@@ -6039,7 +6039,7 @@
         <v>46272.666667</v>
       </c>
       <c r="J62" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K62" s="3">
         <v>272160000.0</v>
@@ -6138,7 +6138,7 @@
         <v>46272.666667</v>
       </c>
       <c r="J63" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K63" s="3">
         <v>927900000.0</v>
@@ -6229,7 +6229,7 @@
         <v>46272.666667</v>
       </c>
       <c r="J64" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K64" s="3">
         <v>30000000.0</v>
@@ -6331,7 +6331,7 @@
         <v>46272.706944</v>
       </c>
       <c r="J65" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K65" s="3">
         <v>1500000.0</v>
@@ -6418,7 +6418,7 @@
         <v>46273.375</v>
       </c>
       <c r="J66" s="0">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K66" s="3"/>
       <c r="L66" s="0" t="inlineStr">
@@ -6524,7 +6524,7 @@
         <v>46273.416667</v>
       </c>
       <c r="J67" s="0">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K67" s="3">
         <v>124000000.0</v>
@@ -6623,7 +6623,7 @@
         <v>46273.625694</v>
       </c>
       <c r="J68" s="0">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K68" s="3"/>
       <c r="L68" s="0" t="inlineStr">
@@ -6714,7 +6714,7 @@
         <v>46273.645833</v>
       </c>
       <c r="J69" s="0">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K69" s="3">
         <v>19980000.0</v>
@@ -6809,7 +6809,7 @@
         <v>46273.645833</v>
       </c>
       <c r="J70" s="0">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K70" s="3">
         <v>52270.0</v>
@@ -6900,7 +6900,7 @@
         <v>46273.666667</v>
       </c>
       <c r="J71" s="0">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K71" s="3"/>
       <c r="L71" s="0" t="inlineStr">
@@ -6997,7 +6997,7 @@
         <v>46274.463194</v>
       </c>
       <c r="J72" s="0">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K72" s="3"/>
       <c r="L72" s="0" t="inlineStr">
@@ -7090,7 +7090,7 @@
         <v>46274.5</v>
       </c>
       <c r="J73" s="0">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K73" s="3">
         <v>7167631.0</v>
@@ -7185,7 +7185,7 @@
         <v>46274.625</v>
       </c>
       <c r="J74" s="0">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K74" s="3">
         <v>1800000.0</v>
@@ -7272,7 +7272,7 @@
         <v>46274.625</v>
       </c>
       <c r="J75" s="0">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K75" s="3">
         <v>30754000.0</v>
@@ -7365,7 +7365,7 @@
         <v>46274.645833</v>
       </c>
       <c r="J76" s="0">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K76" s="3">
         <v>180329688.0</v>
@@ -7460,7 +7460,7 @@
         <v>46274.666667</v>
       </c>
       <c r="J77" s="0">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K77" s="3">
         <v>232851.0</v>
@@ -7555,7 +7555,7 @@
         <v>46275.5</v>
       </c>
       <c r="J78" s="0">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K78" s="3"/>
       <c r="L78" s="0" t="inlineStr">
@@ -7644,7 +7644,7 @@
         <v>46275.625</v>
       </c>
       <c r="J79" s="0">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K79" s="3">
         <v>240000000.0</v>
@@ -7739,7 +7739,7 @@
         <v>46275.625</v>
       </c>
       <c r="J80" s="0">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K80" s="3">
         <v>26000000.0</v>
@@ -7834,7 +7834,7 @@
         <v>46275.666667</v>
       </c>
       <c r="J81" s="0">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K81" s="3"/>
       <c r="L81" s="0" t="inlineStr">
@@ -7927,7 +7927,7 @@
         <v>46276.625</v>
       </c>
       <c r="J82" s="0">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K82" s="3"/>
       <c r="L82" s="0" t="inlineStr">
@@ -8020,7 +8020,7 @@
         <v>46276.666667</v>
       </c>
       <c r="J83" s="0">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K83" s="3"/>
       <c r="L83" s="0" t="inlineStr">
@@ -8113,7 +8113,7 @@
         <v>46276.666667</v>
       </c>
       <c r="J84" s="0">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K84" s="3"/>
       <c r="L84" s="0" t="inlineStr">
@@ -8210,7 +8210,7 @@
         <v>46279.625</v>
       </c>
       <c r="J85" s="0">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K85" s="3">
         <v>540000000.0</v>
@@ -8305,7 +8305,7 @@
         <v>46279.625</v>
       </c>
       <c r="J86" s="0">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K86" s="3"/>
       <c r="L86" s="0" t="inlineStr">
@@ -8396,7 +8396,7 @@
         <v>46279.625</v>
       </c>
       <c r="J87" s="0">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K87" s="3"/>
       <c r="L87" s="0" t="inlineStr">
@@ -8485,7 +8485,7 @@
         <v>46279.666667</v>
       </c>
       <c r="J88" s="0">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K88" s="3">
         <v>225000000.0</v>
@@ -8580,7 +8580,7 @@
         <v>46280.458333</v>
       </c>
       <c r="J89" s="0">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K89" s="3">
         <v>163000000.0</v>
@@ -8677,7 +8677,7 @@
         <v>46280.5</v>
       </c>
       <c r="J90" s="0">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K90" s="3">
         <v>132232000.0</v>
@@ -8768,7 +8768,7 @@
         <v>46280.625</v>
       </c>
       <c r="J91" s="0">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K91" s="3">
         <v>295121.0</v>
@@ -8867,7 +8867,7 @@
         <v>46280.6375</v>
       </c>
       <c r="J92" s="0">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K92" s="3"/>
       <c r="L92" s="0" t="inlineStr">
@@ -8960,7 +8960,7 @@
         <v>46281.583333</v>
       </c>
       <c r="J93" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K93" s="3">
         <v>204000000.0</v>
@@ -9051,7 +9051,7 @@
         <v>46281.729167</v>
       </c>
       <c r="J94" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K94" s="3">
         <v>388644480.0</v>
@@ -9146,7 +9146,7 @@
         <v>46282.375</v>
       </c>
       <c r="J95" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K95" s="3">
         <v>80000000.0</v>
@@ -9241,7 +9241,7 @@
         <v>46282.4375</v>
       </c>
       <c r="J96" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K96" s="3">
         <v>177000000.0</v>
@@ -9336,7 +9336,7 @@
         <v>46286.625694</v>
       </c>
       <c r="J97" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K97" s="3">
         <v>453590167.0</v>
@@ -9427,7 +9427,7 @@
         <v>46286.645833</v>
       </c>
       <c r="J98" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K98" s="3"/>
       <c r="L98" s="0" t="inlineStr">
@@ -9516,7 +9516,7 @@
         <v>46286.666667</v>
       </c>
       <c r="J99" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K99" s="3"/>
       <c r="L99" s="0" t="inlineStr">
@@ -9612,7 +9612,7 @@
         <v>46287.625</v>
       </c>
       <c r="J100" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K100" s="3">
         <v>366678654.0</v>
@@ -9708,7 +9708,7 @@
         <v>46287.625</v>
       </c>
       <c r="J101" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K101" s="3"/>
       <c r="L101" s="0" t="inlineStr">
@@ -9801,7 +9801,7 @@
         <v>46287.625694</v>
       </c>
       <c r="J102" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K102" s="3">
         <v>10000000.0</v>
@@ -9896,7 +9896,7 @@
         <v>46289.625</v>
       </c>
       <c r="J103" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K103" s="3"/>
       <c r="L103" s="0" t="inlineStr">
@@ -9992,7 +9992,7 @@
         <v>46289.729167</v>
       </c>
       <c r="J104" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K104" s="3">
         <v>414000000.0</v>
@@ -10089,7 +10089,7 @@
         <v>46290.625</v>
       </c>
       <c r="J105" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K105" s="3"/>
       <c r="L105" s="0" t="inlineStr">
@@ -10182,7 +10182,7 @@
         <v>46293.645833</v>
       </c>
       <c r="J106" s="0">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K106" s="3">
         <v>450000000.0</v>
@@ -10277,7 +10277,7 @@
         <v>46295.625</v>
       </c>
       <c r="J107" s="0">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K107" s="3">
         <v>24000.0</v>
@@ -10377,7 +10377,7 @@
         <v>46297.625</v>
       </c>
       <c r="J108" s="0">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K108" s="3">
         <v>565250.0</v>

</xml_diff>

<commit_message>
Radar: datos del 2026-09-01
</commit_message>
<xml_diff>
--- a/web/descargas/licitaciones.xlsx
+++ b/web/descargas/licitaciones.xlsx
@@ -219,95 +219,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2422-149-L126</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SOL. 945841, SERVISIO DE FABRICACION E INSTALACION DE TABLERO PARA BALNEARIO</t>
-        </is>
-      </c>
-      <c r="C2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Publicada</t>
-        </is>
-      </c>
-      <c r="D2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">I MUNICIPALIDAD DE PUENTE ALTO</t>
-        </is>
-      </c>
-      <c r="E2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">I MUNICIPALIDAD DE PUENTE ALTO</t>
-        </is>
-      </c>
-      <c r="F2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Región Metropolitana de Santiago</t>
-        </is>
-      </c>
-      <c r="G2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Puente Alto</t>
-        </is>
-      </c>
-      <c r="H2" s="2">
-        <v>46265.753669</v>
-      </c>
-      <c r="I2" s="2">
-        <v>46272.65</v>
-      </c>
-      <c r="J2" s="0">
-        <v>6</v>
-      </c>
-      <c r="K2" s="3">
-        <v>4000000.0</v>
-      </c>
-      <c r="L2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CLP</t>
-        </is>
-      </c>
-      <c r="M2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">L1</t>
-        </is>
-      </c>
-      <c r="N2" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Servicios de producción y fabricación industrial / Fabricación de maquinarias y equipos de transporte / Fabricación de maquinarias</t>
-        </is>
-      </c>
-      <c r="O2" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1 Kit · Servicios de fabricación de calderas para central eléctrica</t>
-        </is>
-      </c>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="0"/>
-      <c r="S2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
-        </is>
-      </c>
-      <c r="T2" s="4"/>
-      <c r="U2" s="0"/>
-      <c r="V2" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NECESIDAD DE SERVICIO, PARA ACONDICIONAMIENTO DE AMBIENTE DE LA PISCINA TEMPERADA BALNEARIO MUNICIPAL, SE REQUIERE SERVICIO DE FABRICACION, INSTALACION Y PUESTA EN MARCHA DE TABLERO DE FUERZA Y COMANDO DE MOTOR TRIFASICO.</t>
-        </is>
-      </c>
-      <c r="W2" s="5" t="str">
-        <f>HYPERLINK("https://www.mercadopublico.cl/Procurement/Modules/RFB/DetailsAcquisition.aspx?idlicitacion=2422-149-L126","descargar bases")</f>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:W2"/>
+  <autoFilter ref="A1:W1"/>
 </worksheet>
 </file>
 

</xml_diff>